<commit_message>
Changed CH card to 6 layer. Added single pt grnd.
CH card is now layed out cleanly with 6 layers.
Added a single point connection with surge protection to the backplane.
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v5/Backplane/Backplane_Slots_BOM_digikey.xlsx
+++ b/Lasser_Driver_v5/Backplane/Backplane_Slots_BOM_digikey.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,6 +633,111 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>RC0805JR-070RL</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Backplane R1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0R</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>R_0805_2012Metric_Pad1.20x1.40mm_HandSolder</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0 ohm single-point net-tie, GND&lt;-&gt;PGND_TEC ground bond</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CL21B104KBCNNNC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Samsung Electro-Mechanics</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Backplane C1</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>100nF</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>C_0805_2012Metric_Pad1.18x1.45mm_HandSolder</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>100nF 50V X7R AC bypass across GND&lt;-&gt;PGND_TEC bond</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SMAJ5.0CA-E3/61</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Vishay General Semiconductor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Backplane D3</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>SMAJ5.0CA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>D_SMA-SMB_Universal_Handsoldering</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Bidirectional 5V TVS (DO-214AC/SMA), transient/fault clamp on GND&lt;-&gt;PGND_TEC bond</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>